<commit_message>
Daily EOD data and reports for 2026-08-12
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260812.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260812.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.58</v>
+        <v>1.57</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-1.25%</t>
+          <t>-1.87%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>242025.98</v>
+        <v>240494.17</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-3063.62</v>
+        <v>-4595.43</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.335</v>
+        <v>2.36</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.035</v>
+        <v>-0.01</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-1.48%</t>
+          <t>-0.42%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>163450</v>
+        <v>165200</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-2450</v>
+        <v>-700</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1.225</v>
+        <v>1.235</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3.38%</t>
+          <t>4.22%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>70386.05</v>
+        <v>70960.63</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>2298.32</v>
+        <v>2872.9</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>63.63</v>
+        <v>63.45</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.3</v>
+        <v>-0.48</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-0.47%</t>
+          <t>-0.75%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>704065.95</v>
+        <v>702074.25</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-3319.5</v>
+        <v>-5311.2</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>173.76</v>
+        <v>172.72</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.16</v>
+        <v>-1.2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.09%</t>
+          <t>-0.69%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.91</v>
+        <v>0.905</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.02</v>
+        <v>0.015</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.25%</t>
+          <t>1.69%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>9100</v>
+        <v>9050</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>137.06</v>
+        <v>138.44</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-1.27</v>
+        <v>0.11</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.92%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>548240</v>
+        <v>553760</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-5080</v>
+        <v>440</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.28</v>
+        <v>0.275</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0</v>
+        <v>-0.005</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-1.79%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>5600</v>
+        <v>5500</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.1</v>
+        <v>0.105</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>941.2</v>
+        <v>988.26</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0</v>
+        <v>47.06</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.099</v>
+        <v>0.001</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>1.01%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-594</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>35.56</v>
+        <v>35.37</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.13</v>
+        <v>-0.32</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.36%</t>
+          <t>-0.90%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.73</v>
+        <v>32.78</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.23</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-0.85%</t>
+          <t>-0.70%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42156.24</v>
+        <v>42220.64</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-360.64</v>
+        <v>-296.24</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1786097.69</v>
+        <v>1790980.22</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-13813.53</v>
+        <v>-8931</v>
       </c>
     </row>
   </sheetData>

</xml_diff>